<commit_message>
Site guncellemesi - 14.09.2026 08:52
</commit_message>
<xml_diff>
--- a/app/mevduat-kredi-faizleri/data/hoca-ile-borsa-faiz-takip-sablonu-guncel.xlsx
+++ b/app/mevduat-kredi-faizleri/data/hoca-ile-borsa-faiz-takip-sablonu-guncel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projeler\hoca-ile-borsa\app\mevduat-kredi-faizleri\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD42B534-2A0E-4681-8691-0CD9F64A716D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F1D15DA-D296-432E-A617-0F653630A77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -655,6 +655,9 @@
                 <c:pt idx="103">
                   <c:v>46276</c:v>
                 </c:pt>
+                <c:pt idx="104">
+                  <c:v>46279</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -977,7 +980,7 @@
                   <c:v>41.642173913043479</c:v>
                 </c:pt>
                 <c:pt idx="104">
-                  <c:v>0</c:v>
+                  <c:v>41.322608695652171</c:v>
                 </c:pt>
                 <c:pt idx="105">
                   <c:v>0</c:v>
@@ -2293,6 +2296,9 @@
                 <c:pt idx="103">
                   <c:v>46276</c:v>
                 </c:pt>
+                <c:pt idx="104">
+                  <c:v>46279</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -2615,7 +2621,7 @@
                   <c:v>3.6068421052631581</c:v>
                 </c:pt>
                 <c:pt idx="104">
-                  <c:v>0</c:v>
+                  <c:v>3.4747368421052629</c:v>
                 </c:pt>
                 <c:pt idx="105">
                   <c:v>0</c:v>
@@ -3931,6 +3937,9 @@
                 <c:pt idx="103">
                   <c:v>46276</c:v>
                 </c:pt>
+                <c:pt idx="104">
+                  <c:v>46279</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -4253,7 +4262,7 @@
                   <c:v>3.0133333333333336</c:v>
                 </c:pt>
                 <c:pt idx="104">
-                  <c:v>0</c:v>
+                  <c:v>3.0022222222222221</c:v>
                 </c:pt>
                 <c:pt idx="105">
                   <c:v>0</c:v>
@@ -5569,6 +5578,9 @@
                 <c:pt idx="103">
                   <c:v>46276</c:v>
                 </c:pt>
+                <c:pt idx="104">
+                  <c:v>46279</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -5891,7 +5903,7 @@
                   <c:v>3.3109999999999999</c:v>
                 </c:pt>
                 <c:pt idx="104">
-                  <c:v>0</c:v>
+                  <c:v>3.3109999999999999</c:v>
                 </c:pt>
                 <c:pt idx="105">
                   <c:v>0</c:v>
@@ -15522,33 +15534,81 @@
       </c>
     </row>
     <row r="109" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A109" s="2"/>
-      <c r="B109" s="3"/>
-      <c r="C109" s="3"/>
-      <c r="D109" s="3"/>
-      <c r="E109" s="3"/>
-      <c r="F109" s="3"/>
-      <c r="G109" s="3"/>
-      <c r="H109" s="3"/>
-      <c r="I109" s="3"/>
-      <c r="J109" s="3"/>
-      <c r="K109" s="3"/>
-      <c r="L109" s="3"/>
-      <c r="M109" s="3"/>
-      <c r="N109" s="3"/>
-      <c r="O109" s="3"/>
-      <c r="P109" s="3"/>
-      <c r="Q109" s="3"/>
-      <c r="R109" s="3"/>
-      <c r="S109" s="3"/>
-      <c r="T109" s="3"/>
-      <c r="U109" s="3"/>
-      <c r="V109" s="3"/>
-      <c r="W109" s="3"/>
-      <c r="X109" s="3"/>
-      <c r="Y109" s="4" t="str">
+      <c r="A109" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B109" s="3">
+        <v>39</v>
+      </c>
+      <c r="C109" s="3">
+        <v>44</v>
+      </c>
+      <c r="D109" s="3">
+        <v>44</v>
+      </c>
+      <c r="E109" s="3">
+        <v>42</v>
+      </c>
+      <c r="F109" s="3">
+        <v>43</v>
+      </c>
+      <c r="G109" s="3">
+        <v>37.75</v>
+      </c>
+      <c r="H109" s="3">
+        <v>44</v>
+      </c>
+      <c r="I109" s="3">
+        <v>38.5</v>
+      </c>
+      <c r="J109" s="3">
+        <v>42</v>
+      </c>
+      <c r="K109" s="3">
+        <v>38</v>
+      </c>
+      <c r="L109" s="3">
+        <v>36</v>
+      </c>
+      <c r="M109" s="3">
+        <v>41</v>
+      </c>
+      <c r="N109" s="3">
+        <v>44</v>
+      </c>
+      <c r="O109" s="3">
+        <v>41.17</v>
+      </c>
+      <c r="P109" s="3">
+        <v>37</v>
+      </c>
+      <c r="Q109" s="3">
+        <v>43</v>
+      </c>
+      <c r="R109" s="3">
+        <v>43.5</v>
+      </c>
+      <c r="S109" s="3">
+        <v>42</v>
+      </c>
+      <c r="T109" s="3">
+        <v>41</v>
+      </c>
+      <c r="U109" s="3">
+        <v>41.25</v>
+      </c>
+      <c r="V109" s="3">
+        <v>38</v>
+      </c>
+      <c r="W109" s="3">
+        <v>45</v>
+      </c>
+      <c r="X109" s="3">
+        <v>45.25</v>
+      </c>
+      <c r="Y109" s="4">
         <f t="shared" si="26"/>
-        <v/>
+        <v>41.322608695652171</v>
       </c>
     </row>
     <row r="110" spans="1:25" x14ac:dyDescent="0.25">
@@ -30986,29 +31046,69 @@
       </c>
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A109" s="2"/>
-      <c r="B109" s="3"/>
-      <c r="C109" s="3"/>
-      <c r="D109" s="3"/>
-      <c r="E109" s="3"/>
-      <c r="F109" s="3"/>
-      <c r="G109" s="3"/>
-      <c r="H109" s="3"/>
-      <c r="I109" s="3"/>
-      <c r="J109" s="3"/>
-      <c r="K109" s="3"/>
-      <c r="L109" s="3"/>
-      <c r="M109" s="3"/>
-      <c r="N109" s="3"/>
-      <c r="O109" s="3"/>
-      <c r="P109" s="3"/>
-      <c r="Q109" s="3"/>
-      <c r="R109" s="3"/>
-      <c r="S109" s="3"/>
-      <c r="T109" s="3"/>
-      <c r="U109" s="4" t="str">
+      <c r="A109" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B109" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="C109" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="D109" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="E109" s="3">
+        <v>3.64</v>
+      </c>
+      <c r="F109" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="G109" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="H109" s="3">
+        <v>3.09</v>
+      </c>
+      <c r="I109" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="J109" s="3">
+        <v>3.69</v>
+      </c>
+      <c r="K109" s="3">
+        <v>4.05</v>
+      </c>
+      <c r="L109" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="M109" s="3">
+        <v>4.3899999999999997</v>
+      </c>
+      <c r="N109" s="3">
+        <v>3.84</v>
+      </c>
+      <c r="O109" s="3">
+        <v>3.64</v>
+      </c>
+      <c r="P109" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="Q109" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="R109" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="S109" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="T109" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="U109" s="4">
         <f t="shared" si="34"/>
-        <v/>
+        <v>3.4747368421052629</v>
       </c>
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
@@ -42152,19 +42252,39 @@
       </c>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A109" s="2"/>
-      <c r="B109" s="3"/>
-      <c r="C109" s="3"/>
-      <c r="D109" s="3"/>
-      <c r="E109" s="3"/>
-      <c r="F109" s="3"/>
-      <c r="G109" s="3"/>
-      <c r="H109" s="3"/>
-      <c r="I109" s="3"/>
-      <c r="J109" s="3"/>
-      <c r="K109" s="4" t="str">
+      <c r="A109" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B109" s="3">
+        <v>3.15</v>
+      </c>
+      <c r="C109" s="3">
+        <v>3.24</v>
+      </c>
+      <c r="D109" s="3">
+        <v>2.87</v>
+      </c>
+      <c r="E109" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="F109" s="3">
+        <v>2.87</v>
+      </c>
+      <c r="G109" s="3">
+        <v>2.88</v>
+      </c>
+      <c r="H109" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="I109" s="3">
+        <v>2.94</v>
+      </c>
+      <c r="J109" s="3">
+        <v>2.89</v>
+      </c>
+      <c r="K109" s="4">
         <f t="shared" si="34"/>
-        <v/>
+        <v>3.0022222222222221</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
@@ -50815,20 +50935,42 @@
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A109" s="2"/>
-      <c r="B109" s="3"/>
-      <c r="C109" s="3"/>
-      <c r="D109" s="3"/>
-      <c r="E109" s="3"/>
-      <c r="F109" s="3"/>
-      <c r="G109" s="3"/>
-      <c r="H109" s="3"/>
-      <c r="I109" s="3"/>
-      <c r="J109" s="3"/>
-      <c r="K109" s="3"/>
-      <c r="L109" s="4" t="str">
+      <c r="A109" s="2">
+        <v>46279</v>
+      </c>
+      <c r="B109" s="3">
+        <v>3.18</v>
+      </c>
+      <c r="C109" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="D109" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="E109" s="3">
+        <v>3.59</v>
+      </c>
+      <c r="F109" s="3">
+        <v>3.27</v>
+      </c>
+      <c r="G109" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="H109" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="I109" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="J109" s="3">
+        <v>3.33</v>
+      </c>
+      <c r="K109" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="L109" s="4">
         <f t="shared" si="34"/>
-        <v/>
+        <v>3.3109999999999999</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Site guncellemesi - 21.09.2026 11:02
</commit_message>
<xml_diff>
--- a/app/mevduat-kredi-faizleri/data/hoca-ile-borsa-faiz-takip-sablonu-guncel.xlsx
+++ b/app/mevduat-kredi-faizleri/data/hoca-ile-borsa-faiz-takip-sablonu-guncel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projeler\hoca-ile-borsa\app\mevduat-kredi-faizleri\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202BA8EA-F68C-4CB7-9B9F-80275C32E311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78034774-48DA-44DE-B8FD-E47742AF7566}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -670,6 +670,9 @@
                 <c:pt idx="108">
                   <c:v>46283</c:v>
                 </c:pt>
+                <c:pt idx="109">
+                  <c:v>46286</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -1007,7 +1010,7 @@
                   <c:v>41.322608695652171</c:v>
                 </c:pt>
                 <c:pt idx="109">
-                  <c:v>0</c:v>
+                  <c:v>39.678260869565221</c:v>
                 </c:pt>
                 <c:pt idx="110">
                   <c:v>0</c:v>
@@ -2323,6 +2326,9 @@
                 <c:pt idx="108">
                   <c:v>46283</c:v>
                 </c:pt>
+                <c:pt idx="109">
+                  <c:v>46286</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -2660,7 +2666,7 @@
                   <c:v>3.4747368421052629</c:v>
                 </c:pt>
                 <c:pt idx="109">
-                  <c:v>0</c:v>
+                  <c:v>3.4610526315789478</c:v>
                 </c:pt>
                 <c:pt idx="110">
                   <c:v>0</c:v>
@@ -3976,6 +3982,9 @@
                 <c:pt idx="108">
                   <c:v>46283</c:v>
                 </c:pt>
+                <c:pt idx="109">
+                  <c:v>46286</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -4313,7 +4322,7 @@
                   <c:v>3.0022222222222221</c:v>
                 </c:pt>
                 <c:pt idx="109">
-                  <c:v>0</c:v>
+                  <c:v>3.0022222222222221</c:v>
                 </c:pt>
                 <c:pt idx="110">
                   <c:v>0</c:v>
@@ -5629,6 +5638,9 @@
                 <c:pt idx="108">
                   <c:v>46283</c:v>
                 </c:pt>
+                <c:pt idx="109">
+                  <c:v>46286</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -5966,7 +5978,7 @@
                   <c:v>3.3109999999999999</c:v>
                 </c:pt>
                 <c:pt idx="109">
-                  <c:v>0</c:v>
+                  <c:v>3.3109999999999999</c:v>
                 </c:pt>
                 <c:pt idx="110">
                   <c:v>0</c:v>
@@ -15972,33 +15984,81 @@
       </c>
     </row>
     <row r="114" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A114" s="2"/>
-      <c r="B114" s="3"/>
-      <c r="C114" s="3"/>
-      <c r="D114" s="3"/>
-      <c r="E114" s="3"/>
-      <c r="F114" s="3"/>
-      <c r="G114" s="3"/>
-      <c r="H114" s="3"/>
-      <c r="I114" s="3"/>
-      <c r="J114" s="3"/>
-      <c r="K114" s="3"/>
-      <c r="L114" s="3"/>
-      <c r="M114" s="3"/>
-      <c r="N114" s="3"/>
-      <c r="O114" s="3"/>
-      <c r="P114" s="3"/>
-      <c r="Q114" s="3"/>
-      <c r="R114" s="3"/>
-      <c r="S114" s="3"/>
-      <c r="T114" s="3"/>
-      <c r="U114" s="3"/>
-      <c r="V114" s="3"/>
-      <c r="W114" s="3"/>
-      <c r="X114" s="3"/>
-      <c r="Y114" s="4" t="str">
+      <c r="A114" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B114" s="3">
+        <v>39</v>
+      </c>
+      <c r="C114" s="3">
+        <v>44</v>
+      </c>
+      <c r="D114" s="3">
+        <v>44</v>
+      </c>
+      <c r="E114" s="3">
+        <v>42</v>
+      </c>
+      <c r="F114" s="3">
+        <v>42</v>
+      </c>
+      <c r="G114" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="H114" s="3">
+        <v>44</v>
+      </c>
+      <c r="I114" s="3">
+        <v>38.5</v>
+      </c>
+      <c r="J114" s="3">
+        <v>41</v>
+      </c>
+      <c r="K114" s="3">
+        <v>38</v>
+      </c>
+      <c r="L114" s="3">
+        <v>36</v>
+      </c>
+      <c r="M114" s="3">
+        <v>41</v>
+      </c>
+      <c r="N114" s="3">
+        <v>44</v>
+      </c>
+      <c r="O114" s="3">
+        <v>41.35</v>
+      </c>
+      <c r="P114" s="3">
+        <v>37</v>
+      </c>
+      <c r="Q114" s="3">
+        <v>42</v>
+      </c>
+      <c r="R114" s="3">
+        <v>43.5</v>
+      </c>
+      <c r="S114" s="3">
+        <v>42</v>
+      </c>
+      <c r="T114" s="3">
+        <v>40.5</v>
+      </c>
+      <c r="U114" s="3">
+        <v>41.75</v>
+      </c>
+      <c r="V114" s="3">
+        <v>38</v>
+      </c>
+      <c r="W114" s="3">
+        <v>44</v>
+      </c>
+      <c r="X114" s="3">
+        <v>45.25</v>
+      </c>
+      <c r="Y114" s="4">
         <f t="shared" si="26"/>
-        <v/>
+        <v>39.678260869565221</v>
       </c>
     </row>
     <row r="115" spans="1:25" x14ac:dyDescent="0.25">
@@ -31616,29 +31676,69 @@
       </c>
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A114" s="2"/>
-      <c r="B114" s="3"/>
-      <c r="C114" s="3"/>
-      <c r="D114" s="3"/>
-      <c r="E114" s="3"/>
-      <c r="F114" s="3"/>
-      <c r="G114" s="3"/>
-      <c r="H114" s="3"/>
-      <c r="I114" s="3"/>
-      <c r="J114" s="3"/>
-      <c r="K114" s="3"/>
-      <c r="L114" s="3"/>
-      <c r="M114" s="3"/>
-      <c r="N114" s="3"/>
-      <c r="O114" s="3"/>
-      <c r="P114" s="3"/>
-      <c r="Q114" s="3"/>
-      <c r="R114" s="3"/>
-      <c r="S114" s="3"/>
-      <c r="T114" s="3"/>
-      <c r="U114" s="4" t="str">
+      <c r="A114" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B114" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="C114" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="D114" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="E114" s="3">
+        <v>3.64</v>
+      </c>
+      <c r="F114" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="G114" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="H114" s="3">
+        <v>3.09</v>
+      </c>
+      <c r="I114" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="J114" s="3">
+        <v>3.69</v>
+      </c>
+      <c r="K114" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="L114" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="M114" s="3">
+        <v>4.3899999999999997</v>
+      </c>
+      <c r="N114" s="3">
+        <v>3.84</v>
+      </c>
+      <c r="O114" s="3">
+        <v>3.64</v>
+      </c>
+      <c r="P114" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="Q114" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="R114" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="S114" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="T114" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="U114" s="4">
         <f t="shared" si="34"/>
-        <v/>
+        <v>3.4610526315789478</v>
       </c>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
@@ -42832,19 +42932,39 @@
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A114" s="2"/>
-      <c r="B114" s="3"/>
-      <c r="C114" s="3"/>
-      <c r="D114" s="3"/>
-      <c r="E114" s="3"/>
-      <c r="F114" s="3"/>
-      <c r="G114" s="3"/>
-      <c r="H114" s="3"/>
-      <c r="I114" s="3"/>
-      <c r="J114" s="3"/>
-      <c r="K114" s="4" t="str">
+      <c r="A114" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B114" s="3">
+        <v>3.15</v>
+      </c>
+      <c r="C114" s="3">
+        <v>3.24</v>
+      </c>
+      <c r="D114" s="3">
+        <v>2.87</v>
+      </c>
+      <c r="E114" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="F114" s="3">
+        <v>2.87</v>
+      </c>
+      <c r="G114" s="3">
+        <v>2.88</v>
+      </c>
+      <c r="H114" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="I114" s="3">
+        <v>2.94</v>
+      </c>
+      <c r="J114" s="3">
+        <v>2.89</v>
+      </c>
+      <c r="K114" s="4">
         <f t="shared" si="34"/>
-        <v/>
+        <v>3.0022222222222221</v>
       </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.25">
@@ -51610,20 +51730,42 @@
       </c>
     </row>
     <row r="114" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A114" s="2"/>
-      <c r="B114" s="3"/>
-      <c r="C114" s="3"/>
-      <c r="D114" s="3"/>
-      <c r="E114" s="3"/>
-      <c r="F114" s="3"/>
-      <c r="G114" s="3"/>
-      <c r="H114" s="3"/>
-      <c r="I114" s="3"/>
-      <c r="J114" s="3"/>
-      <c r="K114" s="3"/>
-      <c r="L114" s="4" t="str">
+      <c r="A114" s="2">
+        <v>46286</v>
+      </c>
+      <c r="B114" s="3">
+        <v>3.18</v>
+      </c>
+      <c r="C114" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="D114" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="E114" s="3">
+        <v>3.59</v>
+      </c>
+      <c r="F114" s="3">
+        <v>3.27</v>
+      </c>
+      <c r="G114" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="H114" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="I114" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="J114" s="3">
+        <v>3.33</v>
+      </c>
+      <c r="K114" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="L114" s="4">
         <f t="shared" si="34"/>
-        <v/>
+        <v>3.3109999999999999</v>
       </c>
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Site guncellemesi - 28.09.2026 09:39
</commit_message>
<xml_diff>
--- a/app/mevduat-kredi-faizleri/data/hoca-ile-borsa-faiz-takip-sablonu-guncel.xlsx
+++ b/app/mevduat-kredi-faizleri/data/hoca-ile-borsa-faiz-takip-sablonu-guncel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projeler\hoca-ile-borsa\app\mevduat-kredi-faizleri\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98828562-F8D4-4725-A23A-60FE0CF7FA7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C4FF2F-19A5-43C6-85F0-C49A1D02B40A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mevduat" sheetId="1" r:id="rId1"/>
@@ -685,6 +685,9 @@
                 <c:pt idx="113">
                   <c:v>46290</c:v>
                 </c:pt>
+                <c:pt idx="114">
+                  <c:v>46293</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -1037,7 +1040,7 @@
                   <c:v>39.678260869565221</c:v>
                 </c:pt>
                 <c:pt idx="114">
-                  <c:v>0</c:v>
+                  <c:v>41.098260869565216</c:v>
                 </c:pt>
                 <c:pt idx="115">
                   <c:v>0</c:v>
@@ -2353,6 +2356,9 @@
                 <c:pt idx="113">
                   <c:v>46290</c:v>
                 </c:pt>
+                <c:pt idx="114">
+                  <c:v>46293</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -2705,7 +2711,7 @@
                   <c:v>3.4610526315789478</c:v>
                 </c:pt>
                 <c:pt idx="114">
-                  <c:v>0</c:v>
+                  <c:v>3.453157894736842</c:v>
                 </c:pt>
                 <c:pt idx="115">
                   <c:v>0</c:v>
@@ -4021,6 +4027,9 @@
                 <c:pt idx="113">
                   <c:v>46290</c:v>
                 </c:pt>
+                <c:pt idx="114">
+                  <c:v>46293</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -4373,7 +4382,7 @@
                   <c:v>3.0022222222222221</c:v>
                 </c:pt>
                 <c:pt idx="114">
-                  <c:v>0</c:v>
+                  <c:v>3.0022222222222221</c:v>
                 </c:pt>
                 <c:pt idx="115">
                   <c:v>0</c:v>
@@ -5689,6 +5698,9 @@
                 <c:pt idx="113">
                   <c:v>46290</c:v>
                 </c:pt>
+                <c:pt idx="114">
+                  <c:v>46293</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:cat>
@@ -6041,7 +6053,7 @@
                   <c:v>3.3109999999999999</c:v>
                 </c:pt>
                 <c:pt idx="114">
-                  <c:v>0</c:v>
+                  <c:v>3.3109999999999999</c:v>
                 </c:pt>
                 <c:pt idx="115">
                   <c:v>0</c:v>
@@ -16422,33 +16434,81 @@
       </c>
     </row>
     <row r="119" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A119" s="2"/>
-      <c r="B119" s="3"/>
-      <c r="C119" s="3"/>
-      <c r="D119" s="3"/>
-      <c r="E119" s="3"/>
-      <c r="F119" s="3"/>
-      <c r="G119" s="3"/>
-      <c r="H119" s="3"/>
-      <c r="I119" s="3"/>
-      <c r="J119" s="3"/>
-      <c r="K119" s="3"/>
-      <c r="L119" s="3"/>
-      <c r="M119" s="3"/>
-      <c r="N119" s="3"/>
-      <c r="O119" s="3"/>
-      <c r="P119" s="3"/>
-      <c r="Q119" s="3"/>
-      <c r="R119" s="3"/>
-      <c r="S119" s="3"/>
-      <c r="T119" s="3"/>
-      <c r="U119" s="3"/>
-      <c r="V119" s="3"/>
-      <c r="W119" s="3"/>
-      <c r="X119" s="3"/>
-      <c r="Y119" s="4" t="str">
+      <c r="A119" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B119" s="3">
+        <v>39</v>
+      </c>
+      <c r="C119" s="3">
+        <v>44</v>
+      </c>
+      <c r="D119" s="3">
+        <v>44</v>
+      </c>
+      <c r="E119" s="3">
+        <v>42</v>
+      </c>
+      <c r="F119" s="3">
+        <v>42</v>
+      </c>
+      <c r="G119" s="3">
+        <v>37.75</v>
+      </c>
+      <c r="H119" s="3">
+        <v>44</v>
+      </c>
+      <c r="I119" s="3">
+        <v>38</v>
+      </c>
+      <c r="J119" s="3">
+        <v>41</v>
+      </c>
+      <c r="K119" s="3">
+        <v>38</v>
+      </c>
+      <c r="L119" s="3">
+        <v>36</v>
+      </c>
+      <c r="M119" s="3">
+        <v>41</v>
+      </c>
+      <c r="N119" s="3">
+        <v>44</v>
+      </c>
+      <c r="O119" s="3">
+        <v>41.26</v>
+      </c>
+      <c r="P119" s="3">
+        <v>38</v>
+      </c>
+      <c r="Q119" s="3">
+        <v>42</v>
+      </c>
+      <c r="R119" s="3">
+        <v>42.5</v>
+      </c>
+      <c r="S119" s="3">
+        <v>42</v>
+      </c>
+      <c r="T119" s="3">
+        <v>40.25</v>
+      </c>
+      <c r="U119" s="3">
+        <v>42</v>
+      </c>
+      <c r="V119" s="3">
+        <v>38</v>
+      </c>
+      <c r="W119" s="3">
+        <v>44</v>
+      </c>
+      <c r="X119" s="3">
+        <v>44.5</v>
+      </c>
+      <c r="Y119" s="4">
         <f t="shared" si="26"/>
-        <v/>
+        <v>41.098260869565216</v>
       </c>
     </row>
     <row r="120" spans="1:25" x14ac:dyDescent="0.25">
@@ -32246,29 +32306,69 @@
       </c>
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A119" s="2"/>
-      <c r="B119" s="3"/>
-      <c r="C119" s="3"/>
-      <c r="D119" s="3"/>
-      <c r="E119" s="3"/>
-      <c r="F119" s="3"/>
-      <c r="G119" s="3"/>
-      <c r="H119" s="3"/>
-      <c r="I119" s="3"/>
-      <c r="J119" s="3"/>
-      <c r="K119" s="3"/>
-      <c r="L119" s="3"/>
-      <c r="M119" s="3"/>
-      <c r="N119" s="3"/>
-      <c r="O119" s="3"/>
-      <c r="P119" s="3"/>
-      <c r="Q119" s="3"/>
-      <c r="R119" s="3"/>
-      <c r="S119" s="3"/>
-      <c r="T119" s="3"/>
-      <c r="U119" s="4" t="str">
+      <c r="A119" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B119" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="C119" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="D119" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="E119" s="3">
+        <v>3.64</v>
+      </c>
+      <c r="F119" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="G119" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="H119" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="I119" s="3">
+        <v>3.14</v>
+      </c>
+      <c r="J119" s="3">
+        <v>3.69</v>
+      </c>
+      <c r="K119" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="L119" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="M119" s="3">
+        <v>4.3899999999999997</v>
+      </c>
+      <c r="N119" s="3">
+        <v>3.84</v>
+      </c>
+      <c r="O119" s="3">
+        <v>3.64</v>
+      </c>
+      <c r="P119" s="3">
+        <v>3.79</v>
+      </c>
+      <c r="Q119" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="R119" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="S119" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="T119" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="U119" s="4">
         <f t="shared" si="34"/>
-        <v/>
+        <v>3.453157894736842</v>
       </c>
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
@@ -43512,19 +43612,39 @@
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A119" s="2"/>
-      <c r="B119" s="3"/>
-      <c r="C119" s="3"/>
-      <c r="D119" s="3"/>
-      <c r="E119" s="3"/>
-      <c r="F119" s="3"/>
-      <c r="G119" s="3"/>
-      <c r="H119" s="3"/>
-      <c r="I119" s="3"/>
-      <c r="J119" s="3"/>
-      <c r="K119" s="4" t="str">
+      <c r="A119" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B119" s="3">
+        <v>3.15</v>
+      </c>
+      <c r="C119" s="3">
+        <v>3.24</v>
+      </c>
+      <c r="D119" s="3">
+        <v>2.87</v>
+      </c>
+      <c r="E119" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="F119" s="3">
+        <v>2.87</v>
+      </c>
+      <c r="G119" s="3">
+        <v>2.88</v>
+      </c>
+      <c r="H119" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="I119" s="3">
+        <v>2.94</v>
+      </c>
+      <c r="J119" s="3">
+        <v>2.89</v>
+      </c>
+      <c r="K119" s="4">
         <f t="shared" si="34"/>
-        <v/>
+        <v>3.0022222222222221</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
@@ -52405,20 +52525,42 @@
       </c>
     </row>
     <row r="119" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A119" s="2"/>
-      <c r="B119" s="3"/>
-      <c r="C119" s="3"/>
-      <c r="D119" s="3"/>
-      <c r="E119" s="3"/>
-      <c r="F119" s="3"/>
-      <c r="G119" s="3"/>
-      <c r="H119" s="3"/>
-      <c r="I119" s="3"/>
-      <c r="J119" s="3"/>
-      <c r="K119" s="3"/>
-      <c r="L119" s="4" t="str">
+      <c r="A119" s="2">
+        <v>46293</v>
+      </c>
+      <c r="B119" s="3">
+        <v>3.18</v>
+      </c>
+      <c r="C119" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="D119" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="E119" s="3">
+        <v>3.59</v>
+      </c>
+      <c r="F119" s="3">
+        <v>3.27</v>
+      </c>
+      <c r="G119" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="H119" s="3">
+        <v>3.19</v>
+      </c>
+      <c r="I119" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="J119" s="3">
+        <v>3.33</v>
+      </c>
+      <c r="K119" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="L119" s="4">
         <f t="shared" si="34"/>
-        <v/>
+        <v>3.3109999999999999</v>
       </c>
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>